<commit_message>
EntityData 新增 SplashRadius（攻击溅射半径）：xlsx 提取 + AttributeStore 全链路接入
- EntityData：SplashRadius float 字段，位于 TargetPriority 与 MaxHp 之间
- XLSX2DataAsset：照 float 字段模板提取 SplashRadius；Rebuild 批处理模式跳过确认框（DisplayDialog 批处理下不可用）
- EntityStats：SetBase 注入 store + 计算属性 SplashRadiusS（无 clamp，同 VisionRadiusS）
- Modifier：float 属性文档清单补 SplashRadius（AddFlat/AddPercent 叠加）
- 测试：base 透传 + AddFlat/AddPercent 修饰 + 按 group 精确移除还原
- 数值接入即完成；选取/触发时机待设计讨论后实现

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Assets/DataTools/EntityAttributes.xlsx
+++ b/Assets/DataTools/EntityAttributes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Unity\projects\TD\Assets\DataTools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEEE6321-0170-45AA-92A6-790BD8D26E88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FECE7746-8601-4AA3-B3B4-AB24A49314A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$4:$BC$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$4:$BD$4</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="442">
   <si>
     <t>ChineseName</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -5959,8 +5959,16 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>_1</t>
-    </r>
+      <t>_skin1</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>溅射半径</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SplashRadius</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -6505,7 +6513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BG34"/>
+  <dimension ref="A1:BH34"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.58203125" style="9" customWidth="1"/>
@@ -6520,22 +6528,22 @@
     <col min="20" max="20" width="12.58203125" style="12" customWidth="1"/>
     <col min="21" max="23" width="12.58203125" style="13" customWidth="1"/>
     <col min="24" max="26" width="12.58203125" style="11" customWidth="1"/>
-    <col min="27" max="31" width="12.58203125" style="13" customWidth="1"/>
-    <col min="32" max="40" width="12.58203125" style="11" customWidth="1"/>
-    <col min="41" max="41" width="12.58203125" style="12" customWidth="1"/>
-    <col min="42" max="43" width="12.58203125" style="11" customWidth="1"/>
-    <col min="44" max="47" width="12.58203125" style="10" customWidth="1"/>
-    <col min="48" max="49" width="12.58203125" style="14" customWidth="1"/>
-    <col min="50" max="50" width="12.58203125" style="10" customWidth="1"/>
-    <col min="51" max="51" width="12.58203125" style="14" customWidth="1"/>
-    <col min="52" max="52" width="12.58203125" style="10" customWidth="1"/>
-    <col min="53" max="53" width="12.58203125" style="13" customWidth="1"/>
-    <col min="54" max="55" width="12.58203125" style="11" customWidth="1"/>
-    <col min="56" max="58" width="12.58203125" style="4" customWidth="1"/>
-    <col min="59" max="16384" width="8.6640625" style="7"/>
+    <col min="27" max="32" width="12.58203125" style="13" customWidth="1"/>
+    <col min="33" max="41" width="12.58203125" style="11" customWidth="1"/>
+    <col min="42" max="42" width="12.58203125" style="12" customWidth="1"/>
+    <col min="43" max="44" width="12.58203125" style="11" customWidth="1"/>
+    <col min="45" max="48" width="12.58203125" style="10" customWidth="1"/>
+    <col min="49" max="50" width="12.58203125" style="14" customWidth="1"/>
+    <col min="51" max="51" width="12.58203125" style="10" customWidth="1"/>
+    <col min="52" max="52" width="12.58203125" style="14" customWidth="1"/>
+    <col min="53" max="53" width="12.58203125" style="10" customWidth="1"/>
+    <col min="54" max="54" width="12.58203125" style="13" customWidth="1"/>
+    <col min="55" max="56" width="12.58203125" style="11" customWidth="1"/>
+    <col min="57" max="59" width="12.58203125" style="4" customWidth="1"/>
+    <col min="60" max="16384" width="8.6640625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>2</v>
       </c>
@@ -6598,9 +6606,10 @@
       <c r="BD1" s="6"/>
       <c r="BE1" s="6"/>
       <c r="BF1" s="6"/>
-      <c r="BG1" s="20"/>
+      <c r="BG1" s="6"/>
+      <c r="BH1" s="20"/>
     </row>
-    <row r="2" spans="1:59" ht="14.5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:60" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A2" s="29" t="s">
         <v>4</v>
       </c>
@@ -6652,10 +6661,10 @@
       <c r="AO2" s="6"/>
       <c r="AP2" s="6"/>
       <c r="AQ2" s="6"/>
-      <c r="AR2" s="29" t="s">
+      <c r="AR2" s="6"/>
+      <c r="AS2" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="AS2" s="29"/>
       <c r="AT2" s="29"/>
       <c r="AU2" s="29"/>
       <c r="AV2" s="29"/>
@@ -6663,19 +6672,20 @@
       <c r="AX2" s="29"/>
       <c r="AY2" s="29"/>
       <c r="AZ2" s="29"/>
-      <c r="BA2" s="6" t="s">
+      <c r="BA2" s="29"/>
+      <c r="BB2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="BB2" s="6"/>
       <c r="BC2" s="6"/>
-      <c r="BD2" s="1" t="s">
+      <c r="BD2" s="6"/>
+      <c r="BE2" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="BE2" s="1"/>
       <c r="BF2" s="1"/>
-      <c r="BG2" s="20"/>
+      <c r="BG2" s="1"/>
+      <c r="BH2" s="20"/>
     </row>
-    <row r="3" spans="1:59" s="8" customFormat="1" ht="14.5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:60" s="8" customFormat="1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A3" s="30" t="s">
         <v>73</v>
       </c>
@@ -6754,105 +6764,108 @@
       <c r="Z3" s="33" t="s">
         <v>298</v>
       </c>
-      <c r="AA3" s="32" t="s">
+      <c r="AA3" s="33" t="s">
+        <v>440</v>
+      </c>
+      <c r="AB3" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="AB3" s="32" t="s">
+      <c r="AC3" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="AC3" s="32" t="s">
+      <c r="AD3" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="AD3" s="32" t="s">
+      <c r="AE3" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="AE3" s="32" t="s">
+      <c r="AF3" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="AF3" s="32" t="s">
+      <c r="AG3" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="AG3" s="32" t="s">
+      <c r="AH3" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="AH3" s="33" t="s">
+      <c r="AI3" s="33" t="s">
         <v>180</v>
       </c>
-      <c r="AI3" s="33" t="s">
+      <c r="AJ3" s="33" t="s">
         <v>181</v>
       </c>
-      <c r="AJ3" s="33" t="s">
+      <c r="AK3" s="33" t="s">
         <v>182</v>
       </c>
-      <c r="AK3" s="33" t="s">
+      <c r="AL3" s="33" t="s">
         <v>183</v>
       </c>
-      <c r="AL3" s="33" t="s">
+      <c r="AM3" s="33" t="s">
         <v>184</v>
       </c>
-      <c r="AM3" s="33" t="s">
+      <c r="AN3" s="33" t="s">
         <v>185</v>
       </c>
-      <c r="AN3" s="33" t="s">
+      <c r="AO3" s="33" t="s">
         <v>186</v>
       </c>
-      <c r="AO3" s="32" t="s">
+      <c r="AP3" s="32" t="s">
         <v>82</v>
       </c>
-      <c r="AP3" s="32" t="s">
+      <c r="AQ3" s="32" t="s">
         <v>83</v>
       </c>
-      <c r="AQ3" s="33" t="s">
+      <c r="AR3" s="33" t="s">
         <v>245</v>
       </c>
-      <c r="AR3" s="30" t="s">
+      <c r="AS3" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="AS3" s="30" t="s">
+      <c r="AT3" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="AT3" s="34" t="s">
+      <c r="AU3" s="34" t="s">
         <v>194</v>
       </c>
-      <c r="AU3" s="30" t="s">
+      <c r="AV3" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="AV3" s="30" t="s">
+      <c r="AW3" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="AW3" s="31" t="s">
+      <c r="AX3" s="31" t="s">
         <v>197</v>
       </c>
-      <c r="AX3" s="30" t="s">
+      <c r="AY3" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="AY3" s="30" t="s">
+      <c r="AZ3" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="AZ3" s="30" t="s">
+      <c r="BA3" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="BA3" s="32" t="s">
+      <c r="BB3" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="BB3" s="32" t="s">
+      <c r="BC3" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="BC3" s="32" t="s">
+      <c r="BD3" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="BD3" s="2" t="s">
+      <c r="BE3" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="BE3" s="2" t="s">
+      <c r="BF3" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="BF3" s="2" t="s">
+      <c r="BG3" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="BG3" s="21"/>
+      <c r="BH3" s="21"/>
     </row>
-    <row r="4" spans="1:59" s="8" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:60" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="30" t="s">
         <v>42</v>
       </c>
@@ -6932,104 +6945,107 @@
         <v>297</v>
       </c>
       <c r="AA4" s="32" t="s">
+        <v>441</v>
+      </c>
+      <c r="AB4" s="32" t="s">
         <v>215</v>
       </c>
-      <c r="AB4" s="32" t="s">
+      <c r="AC4" s="32" t="s">
         <v>216</v>
       </c>
-      <c r="AC4" s="32" t="s">
+      <c r="AD4" s="32" t="s">
         <v>217</v>
       </c>
-      <c r="AD4" s="32" t="s">
+      <c r="AE4" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="AE4" s="32" t="s">
+      <c r="AF4" s="32" t="s">
         <v>219</v>
       </c>
-      <c r="AF4" s="32" t="s">
+      <c r="AG4" s="32" t="s">
         <v>220</v>
       </c>
-      <c r="AG4" s="32" t="s">
+      <c r="AH4" s="32" t="s">
         <v>221</v>
       </c>
-      <c r="AH4" s="32" t="s">
+      <c r="AI4" s="32" t="s">
         <v>223</v>
       </c>
-      <c r="AI4" s="32" t="s">
+      <c r="AJ4" s="32" t="s">
         <v>224</v>
       </c>
-      <c r="AJ4" s="32" t="s">
+      <c r="AK4" s="32" t="s">
         <v>225</v>
       </c>
-      <c r="AK4" s="32" t="s">
+      <c r="AL4" s="32" t="s">
         <v>226</v>
       </c>
-      <c r="AL4" s="32" t="s">
+      <c r="AM4" s="32" t="s">
         <v>227</v>
       </c>
-      <c r="AM4" s="32" t="s">
+      <c r="AN4" s="32" t="s">
         <v>228</v>
       </c>
-      <c r="AN4" s="32" t="s">
+      <c r="AO4" s="32" t="s">
         <v>229</v>
       </c>
-      <c r="AO4" s="32" t="s">
+      <c r="AP4" s="32" t="s">
         <v>230</v>
       </c>
-      <c r="AP4" s="32" t="s">
+      <c r="AQ4" s="32" t="s">
         <v>231</v>
       </c>
-      <c r="AQ4" s="32" t="s">
+      <c r="AR4" s="32" t="s">
         <v>244</v>
       </c>
-      <c r="AR4" s="30" t="s">
+      <c r="AS4" s="30" t="s">
         <v>232</v>
       </c>
-      <c r="AS4" s="30" t="s">
+      <c r="AT4" s="30" t="s">
         <v>233</v>
       </c>
-      <c r="AT4" s="30" t="s">
+      <c r="AU4" s="30" t="s">
         <v>234</v>
       </c>
-      <c r="AU4" s="30" t="s">
+      <c r="AV4" s="30" t="s">
         <v>235</v>
       </c>
-      <c r="AV4" s="30" t="s">
+      <c r="AW4" s="30" t="s">
         <v>236</v>
       </c>
-      <c r="AW4" s="30" t="s">
+      <c r="AX4" s="30" t="s">
         <v>237</v>
       </c>
-      <c r="AX4" s="30" t="s">
+      <c r="AY4" s="30" t="s">
         <v>238</v>
       </c>
-      <c r="AY4" s="30" t="s">
+      <c r="AZ4" s="30" t="s">
         <v>239</v>
       </c>
-      <c r="AZ4" s="30" t="s">
+      <c r="BA4" s="30" t="s">
         <v>240</v>
       </c>
-      <c r="BA4" s="32" t="s">
+      <c r="BB4" s="32" t="s">
         <v>241</v>
       </c>
-      <c r="BB4" s="32" t="s">
+      <c r="BC4" s="32" t="s">
         <v>242</v>
       </c>
-      <c r="BC4" s="32" t="s">
+      <c r="BD4" s="32" t="s">
         <v>243</v>
       </c>
-      <c r="BD4" s="3" t="s">
+      <c r="BE4" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="BE4" s="3" t="s">
+      <c r="BF4" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="BF4" s="3" t="s">
+      <c r="BG4" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="BG4" s="21"/>
+      <c r="BH4" s="21"/>
     </row>
-    <row r="5" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
         <v>44</v>
       </c>
@@ -7099,25 +7115,25 @@
         <v>0</v>
       </c>
       <c r="AA5" s="26">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="26">
         <v>1743</v>
       </c>
-      <c r="AB5" s="26">
+      <c r="AC5" s="26">
         <v>122</v>
       </c>
-      <c r="AC5" s="26">
+      <c r="AD5" s="26">
         <v>20</v>
       </c>
-      <c r="AD5" s="26">
-        <v>0</v>
-      </c>
       <c r="AE5" s="26">
         <v>0</v>
       </c>
-      <c r="AF5" s="24">
-        <v>1</v>
+      <c r="AF5" s="26">
+        <v>0</v>
       </c>
       <c r="AG5" s="24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH5" s="24">
         <v>0</v>
@@ -7140,56 +7156,59 @@
       <c r="AN5" s="24">
         <v>0</v>
       </c>
-      <c r="AO5" s="25" t="s">
+      <c r="AO5" s="24">
+        <v>0</v>
+      </c>
+      <c r="AP5" s="25" t="s">
         <v>190</v>
       </c>
-      <c r="AP5" s="24" t="s">
+      <c r="AQ5" s="24" t="s">
         <v>178</v>
       </c>
-      <c r="AQ5" s="24">
-        <v>1</v>
-      </c>
-      <c r="AR5" s="23">
+      <c r="AR5" s="24">
+        <v>1</v>
+      </c>
+      <c r="AS5" s="23">
         <v>19</v>
       </c>
-      <c r="AS5" s="23">
-        <v>1</v>
-      </c>
       <c r="AT5" s="23">
         <v>1</v>
       </c>
       <c r="AU5" s="23">
         <v>1</v>
       </c>
-      <c r="AV5" s="27">
+      <c r="AV5" s="23">
+        <v>1</v>
+      </c>
+      <c r="AW5" s="27">
         <v>70</v>
       </c>
-      <c r="AW5" s="28" t="s">
+      <c r="AX5" s="28" t="s">
         <v>196</v>
       </c>
-      <c r="AX5" s="23">
-        <v>1</v>
-      </c>
-      <c r="AY5" s="27">
+      <c r="AY5" s="23">
+        <v>1</v>
+      </c>
+      <c r="AZ5" s="27">
         <v>50</v>
       </c>
-      <c r="AZ5" s="23">
-        <v>1</v>
-      </c>
-      <c r="BA5" s="26"/>
-      <c r="BB5" s="24"/>
+      <c r="BA5" s="23">
+        <v>1</v>
+      </c>
+      <c r="BB5" s="26"/>
       <c r="BC5" s="24"/>
-      <c r="BD5" s="4" t="s">
+      <c r="BD5" s="24"/>
+      <c r="BE5" s="4" t="s">
         <v>438</v>
       </c>
-      <c r="BE5" s="5" t="s">
+      <c r="BF5" s="5" t="s">
         <v>302</v>
       </c>
-      <c r="BF5" s="4" t="s">
+      <c r="BG5" s="4" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="6" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>46</v>
       </c>
@@ -7254,25 +7273,25 @@
         <v>0</v>
       </c>
       <c r="AA6" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="13">
         <v>1678</v>
       </c>
-      <c r="AB6" s="13">
+      <c r="AC6" s="13">
         <v>135</v>
       </c>
-      <c r="AC6" s="13">
+      <c r="AD6" s="13">
         <v>20</v>
       </c>
-      <c r="AD6" s="13">
-        <v>0</v>
-      </c>
       <c r="AE6" s="13">
         <v>0</v>
       </c>
-      <c r="AF6" s="11">
-        <v>1</v>
+      <c r="AF6" s="13">
+        <v>0</v>
       </c>
       <c r="AG6" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH6" s="11">
         <v>0</v>
@@ -7295,47 +7314,50 @@
       <c r="AN6" s="11">
         <v>0</v>
       </c>
-      <c r="AQ6" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR6" s="10">
+      <c r="AO6" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR6" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS6" s="10">
         <v>23</v>
       </c>
-      <c r="AS6" s="10">
-        <v>1</v>
-      </c>
       <c r="AT6" s="10">
         <v>1</v>
       </c>
       <c r="AU6" s="10">
         <v>1</v>
       </c>
-      <c r="AV6" s="14">
+      <c r="AV6" s="10">
+        <v>1</v>
+      </c>
+      <c r="AW6" s="14">
         <v>66</v>
       </c>
-      <c r="AW6" s="15" t="s">
+      <c r="AX6" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="AX6" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY6" s="14">
+      <c r="AY6" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ6" s="14">
         <v>50</v>
       </c>
-      <c r="AZ6" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD6" s="4" t="s">
+      <c r="BA6" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE6" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="BE6" s="5" t="s">
+      <c r="BF6" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="BF6" s="4" t="s">
+      <c r="BG6" s="4" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="7" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>50</v>
       </c>
@@ -7400,25 +7422,25 @@
         <v>0</v>
       </c>
       <c r="AA7" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="13">
         <v>1060</v>
       </c>
-      <c r="AB7" s="13">
+      <c r="AC7" s="13">
         <v>126</v>
       </c>
-      <c r="AC7" s="13">
-        <v>0</v>
-      </c>
       <c r="AD7" s="13">
         <v>0</v>
       </c>
       <c r="AE7" s="13">
         <v>0</v>
       </c>
-      <c r="AF7" s="11">
-        <v>1</v>
+      <c r="AF7" s="13">
+        <v>0</v>
       </c>
       <c r="AG7" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH7" s="11">
         <v>0</v>
@@ -7441,47 +7463,50 @@
       <c r="AN7" s="11">
         <v>0</v>
       </c>
-      <c r="AQ7" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR7" s="10">
+      <c r="AO7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR7" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS7" s="10">
         <v>9</v>
       </c>
-      <c r="AS7" s="10">
-        <v>1</v>
-      </c>
       <c r="AT7" s="10">
         <v>1</v>
       </c>
       <c r="AU7" s="10">
         <v>1</v>
       </c>
-      <c r="AV7" s="14">
+      <c r="AV7" s="10">
+        <v>1</v>
+      </c>
+      <c r="AW7" s="14">
         <v>66</v>
       </c>
-      <c r="AW7" s="15" t="s">
+      <c r="AX7" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="AX7" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY7" s="14">
+      <c r="AY7" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ7" s="14">
         <v>50</v>
       </c>
-      <c r="AZ7" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD7" s="4" t="s">
+      <c r="BA7" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE7" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="BE7" s="5" t="s">
+      <c r="BF7" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="BF7" s="4" t="s">
+      <c r="BG7" s="4" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="8" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>50</v>
       </c>
@@ -7546,25 +7571,25 @@
         <v>0</v>
       </c>
       <c r="AA8" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="13">
         <v>1100</v>
       </c>
-      <c r="AB8" s="13">
+      <c r="AC8" s="13">
         <v>90</v>
       </c>
-      <c r="AC8" s="13">
+      <c r="AD8" s="13">
         <v>15</v>
       </c>
-      <c r="AD8" s="13">
-        <v>0</v>
-      </c>
       <c r="AE8" s="13">
         <v>0</v>
       </c>
-      <c r="AF8" s="11">
-        <v>1</v>
+      <c r="AF8" s="13">
+        <v>0</v>
       </c>
       <c r="AG8" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH8" s="11">
         <v>0</v>
@@ -7587,47 +7612,50 @@
       <c r="AN8" s="11">
         <v>0</v>
       </c>
-      <c r="AQ8" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR8" s="10">
+      <c r="AO8" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR8" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS8" s="10">
         <v>16</v>
       </c>
-      <c r="AS8" s="10">
-        <v>1</v>
-      </c>
       <c r="AT8" s="10">
         <v>1</v>
       </c>
       <c r="AU8" s="10">
         <v>1</v>
       </c>
-      <c r="AV8" s="14">
+      <c r="AV8" s="10">
+        <v>1</v>
+      </c>
+      <c r="AW8" s="14">
         <v>60</v>
       </c>
-      <c r="AW8" s="15" t="s">
+      <c r="AX8" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="AX8" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY8" s="14">
+      <c r="AY8" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ8" s="14">
         <v>50</v>
       </c>
-      <c r="AZ8" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD8" s="4" t="s">
+      <c r="BA8" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE8" s="4" t="s">
         <v>272</v>
       </c>
-      <c r="BE8" s="5" t="s">
+      <c r="BF8" s="5" t="s">
         <v>276</v>
       </c>
-      <c r="BF8" s="4" t="s">
+      <c r="BG8" s="4" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="9" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>50</v>
       </c>
@@ -7692,26 +7720,26 @@
         <v>0</v>
       </c>
       <c r="AA9" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB9" s="13">
         <v>1833</v>
       </c>
-      <c r="AB9" s="13">
+      <c r="AC9" s="13">
         <v>496</v>
       </c>
-      <c r="AC9" s="13">
+      <c r="AD9" s="13">
         <v>10</v>
       </c>
-      <c r="AD9" s="13">
-        <v>0</v>
-      </c>
       <c r="AE9" s="13">
         <v>0</v>
       </c>
-      <c r="AF9" s="11">
+      <c r="AF9" s="13">
+        <v>0</v>
+      </c>
+      <c r="AG9" s="11">
         <v>3</v>
       </c>
-      <c r="AG9" s="11">
-        <v>0</v>
-      </c>
       <c r="AH9" s="11">
         <v>0</v>
       </c>
@@ -7733,47 +7761,50 @@
       <c r="AN9" s="11">
         <v>0</v>
       </c>
-      <c r="AQ9" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR9" s="10">
+      <c r="AO9" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR9" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS9" s="10">
         <v>15</v>
       </c>
-      <c r="AS9" s="10">
-        <v>1</v>
-      </c>
       <c r="AT9" s="10">
         <v>1</v>
       </c>
       <c r="AU9" s="10">
-        <v>0</v>
-      </c>
-      <c r="AV9" s="14">
+        <v>1</v>
+      </c>
+      <c r="AV9" s="10">
+        <v>0</v>
+      </c>
+      <c r="AW9" s="14">
         <v>66</v>
       </c>
-      <c r="AW9" s="15" t="s">
+      <c r="AX9" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="AX9" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY9" s="14">
+      <c r="AY9" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ9" s="14">
         <v>50</v>
       </c>
-      <c r="AZ9" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD9" s="4" t="s">
+      <c r="BA9" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE9" s="4" t="s">
         <v>273</v>
       </c>
-      <c r="BE9" s="5" t="s">
+      <c r="BF9" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="BF9" s="4" t="s">
+      <c r="BG9" s="4" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="10" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>50</v>
       </c>
@@ -7838,25 +7869,25 @@
         <v>0</v>
       </c>
       <c r="AA10" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB10" s="13">
         <v>2745</v>
       </c>
-      <c r="AB10" s="13">
+      <c r="AC10" s="13">
         <v>155</v>
       </c>
-      <c r="AC10" s="13">
-        <v>0</v>
-      </c>
       <c r="AD10" s="13">
         <v>0</v>
       </c>
       <c r="AE10" s="13">
         <v>0</v>
       </c>
-      <c r="AF10" s="11">
-        <v>1</v>
+      <c r="AF10" s="13">
+        <v>0</v>
       </c>
       <c r="AG10" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH10" s="11">
         <v>0</v>
@@ -7879,47 +7910,50 @@
       <c r="AN10" s="11">
         <v>0</v>
       </c>
-      <c r="AQ10" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR10" s="10">
+      <c r="AO10" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR10" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS10" s="10">
         <v>13</v>
       </c>
-      <c r="AS10" s="10">
-        <v>1</v>
-      </c>
       <c r="AT10" s="10">
         <v>1</v>
       </c>
       <c r="AU10" s="10">
-        <v>0</v>
-      </c>
-      <c r="AV10" s="14">
+        <v>1</v>
+      </c>
+      <c r="AV10" s="10">
+        <v>0</v>
+      </c>
+      <c r="AW10" s="14">
         <v>60</v>
       </c>
-      <c r="AW10" s="15" t="s">
+      <c r="AX10" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="AX10" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY10" s="14">
+      <c r="AY10" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ10" s="14">
         <v>50</v>
       </c>
-      <c r="AZ10" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD10" s="4" t="s">
+      <c r="BA10" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE10" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="BE10" s="5" t="s">
+      <c r="BF10" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="BF10" s="4" t="s">
+      <c r="BG10" s="4" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="11" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>278</v>
       </c>
@@ -7984,25 +8018,25 @@
         <v>2</v>
       </c>
       <c r="AA11" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB11" s="13">
         <v>1220</v>
       </c>
-      <c r="AB11" s="13">
+      <c r="AC11" s="13">
         <v>110</v>
       </c>
-      <c r="AC11" s="13">
-        <v>0</v>
-      </c>
       <c r="AD11" s="13">
         <v>0</v>
       </c>
       <c r="AE11" s="13">
         <v>0</v>
       </c>
-      <c r="AF11" s="11">
-        <v>1</v>
+      <c r="AF11" s="13">
+        <v>0</v>
       </c>
       <c r="AG11" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH11" s="11">
         <v>0</v>
@@ -8025,47 +8059,50 @@
       <c r="AN11" s="11">
         <v>0</v>
       </c>
-      <c r="AQ11" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR11" s="10">
+      <c r="AO11" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR11" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS11" s="10">
         <v>15</v>
       </c>
-      <c r="AS11" s="10">
-        <v>1</v>
-      </c>
       <c r="AT11" s="10">
         <v>1</v>
       </c>
       <c r="AU11" s="10">
         <v>1</v>
       </c>
-      <c r="AV11" s="14">
+      <c r="AV11" s="10">
+        <v>1</v>
+      </c>
+      <c r="AW11" s="14">
         <v>60</v>
       </c>
-      <c r="AW11" s="15" t="s">
+      <c r="AX11" s="15" t="s">
         <v>287</v>
       </c>
-      <c r="AX11" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY11" s="14">
+      <c r="AY11" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ11" s="14">
         <v>50</v>
       </c>
-      <c r="AZ11" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD11" s="4" t="s">
+      <c r="BA11" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE11" s="4" t="s">
         <v>292</v>
       </c>
-      <c r="BE11" s="5" t="s">
+      <c r="BF11" s="5" t="s">
         <v>293</v>
       </c>
-      <c r="BF11" s="4" t="s">
+      <c r="BG11" s="4" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="12" spans="1:59" ht="14" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:60" ht="14" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>304</v>
       </c>
@@ -8130,25 +8167,25 @@
         <v>0</v>
       </c>
       <c r="AA12" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB12" s="13">
         <v>1080</v>
       </c>
-      <c r="AB12" s="13">
+      <c r="AC12" s="13">
         <v>134</v>
       </c>
-      <c r="AC12" s="13">
-        <v>0</v>
-      </c>
       <c r="AD12" s="13">
         <v>0</v>
       </c>
       <c r="AE12" s="13">
         <v>0</v>
       </c>
-      <c r="AF12" s="11">
-        <v>1</v>
+      <c r="AF12" s="13">
+        <v>0</v>
       </c>
       <c r="AG12" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH12" s="11">
         <v>0</v>
@@ -8171,47 +8208,50 @@
       <c r="AN12" s="11">
         <v>0</v>
       </c>
-      <c r="AQ12" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR12" s="10">
+      <c r="AO12" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR12" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS12" s="10">
         <v>9</v>
       </c>
-      <c r="AS12" s="10">
-        <v>1</v>
-      </c>
       <c r="AT12" s="10">
         <v>1</v>
       </c>
       <c r="AU12" s="10">
         <v>1</v>
       </c>
-      <c r="AV12" s="14">
+      <c r="AV12" s="10">
+        <v>1</v>
+      </c>
+      <c r="AW12" s="14">
         <v>60</v>
       </c>
-      <c r="AW12" s="15" t="s">
+      <c r="AX12" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="AX12" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY12" s="14">
+      <c r="AY12" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ12" s="14">
         <v>50</v>
       </c>
-      <c r="AZ12" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD12" s="4" t="s">
+      <c r="BA12" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE12" s="4" t="s">
         <v>376</v>
       </c>
-      <c r="BE12" s="5" t="s">
+      <c r="BF12" s="5" t="s">
         <v>377</v>
       </c>
-      <c r="BF12" s="4" t="s">
+      <c r="BG12" s="4" t="s">
         <v>378</v>
       </c>
     </row>
-    <row r="13" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
         <v>304</v>
       </c>
@@ -8276,25 +8316,25 @@
         <v>2</v>
       </c>
       <c r="AA13" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB13" s="13">
         <v>1135</v>
       </c>
-      <c r="AB13" s="13">
+      <c r="AC13" s="13">
         <v>109</v>
       </c>
-      <c r="AC13" s="13">
-        <v>0</v>
-      </c>
       <c r="AD13" s="13">
         <v>0</v>
       </c>
       <c r="AE13" s="13">
         <v>0</v>
       </c>
-      <c r="AF13" s="11">
-        <v>1</v>
+      <c r="AF13" s="13">
+        <v>0</v>
       </c>
       <c r="AG13" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH13" s="11">
         <v>0</v>
@@ -8317,47 +8357,50 @@
       <c r="AN13" s="11">
         <v>0</v>
       </c>
-      <c r="AQ13" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR13" s="10">
+      <c r="AO13" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR13" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS13" s="10">
         <v>15</v>
       </c>
-      <c r="AS13" s="10">
-        <v>1</v>
-      </c>
       <c r="AT13" s="10">
         <v>1</v>
       </c>
       <c r="AU13" s="10">
         <v>1</v>
       </c>
-      <c r="AV13" s="14">
+      <c r="AV13" s="10">
+        <v>1</v>
+      </c>
+      <c r="AW13" s="14">
         <v>66</v>
       </c>
-      <c r="AW13" s="15" t="s">
+      <c r="AX13" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="AX13" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY13" s="14">
+      <c r="AY13" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ13" s="14">
         <v>50</v>
       </c>
-      <c r="AZ13" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD13" s="4" t="s">
+      <c r="BA13" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE13" s="4" t="s">
         <v>379</v>
       </c>
-      <c r="BE13" s="5" t="s">
+      <c r="BF13" s="5" t="s">
         <v>380</v>
       </c>
-      <c r="BF13" s="4" t="s">
+      <c r="BG13" s="4" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="14" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
         <v>304</v>
       </c>
@@ -8422,26 +8465,26 @@
         <v>0</v>
       </c>
       <c r="AA14" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB14" s="13">
         <v>2630</v>
       </c>
-      <c r="AB14" s="13">
+      <c r="AC14" s="13">
         <v>475</v>
       </c>
-      <c r="AC14" s="13">
-        <v>0</v>
-      </c>
       <c r="AD14" s="13">
         <v>0</v>
       </c>
       <c r="AE14" s="13">
         <v>0</v>
       </c>
-      <c r="AF14" s="11">
+      <c r="AF14" s="13">
+        <v>0</v>
+      </c>
+      <c r="AG14" s="11">
         <v>3</v>
       </c>
-      <c r="AG14" s="11">
-        <v>0</v>
-      </c>
       <c r="AH14" s="11">
         <v>0</v>
       </c>
@@ -8463,47 +8506,50 @@
       <c r="AN14" s="11">
         <v>0</v>
       </c>
-      <c r="AQ14" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR14" s="10">
+      <c r="AO14" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR14" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS14" s="10">
         <v>16</v>
       </c>
-      <c r="AS14" s="10">
-        <v>1</v>
-      </c>
       <c r="AT14" s="10">
         <v>1</v>
       </c>
       <c r="AU14" s="10">
-        <v>0</v>
-      </c>
-      <c r="AV14" s="14">
+        <v>1</v>
+      </c>
+      <c r="AV14" s="10">
+        <v>0</v>
+      </c>
+      <c r="AW14" s="14">
         <v>60</v>
       </c>
-      <c r="AW14" s="15" t="s">
+      <c r="AX14" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="AX14" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY14" s="14">
+      <c r="AY14" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ14" s="14">
         <v>50</v>
       </c>
-      <c r="AZ14" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD14" s="4" t="s">
+      <c r="BA14" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE14" s="4" t="s">
         <v>382</v>
       </c>
-      <c r="BE14" s="5" t="s">
+      <c r="BF14" s="5" t="s">
         <v>383</v>
       </c>
-      <c r="BF14" s="4" t="s">
+      <c r="BG14" s="4" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="15" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
         <v>304</v>
       </c>
@@ -8568,26 +8614,26 @@
         <v>0</v>
       </c>
       <c r="AA15" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB15" s="13">
         <v>2035</v>
       </c>
-      <c r="AB15" s="13">
+      <c r="AC15" s="13">
         <v>578</v>
       </c>
-      <c r="AC15" s="13">
-        <v>0</v>
-      </c>
       <c r="AD15" s="13">
         <v>0</v>
       </c>
       <c r="AE15" s="13">
         <v>0</v>
       </c>
-      <c r="AF15" s="11">
+      <c r="AF15" s="13">
+        <v>0</v>
+      </c>
+      <c r="AG15" s="11">
         <v>3</v>
       </c>
-      <c r="AG15" s="11">
-        <v>0</v>
-      </c>
       <c r="AH15" s="11">
         <v>0</v>
       </c>
@@ -8609,47 +8655,50 @@
       <c r="AN15" s="11">
         <v>0</v>
       </c>
-      <c r="AQ15" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR15" s="10">
+      <c r="AO15" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR15" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS15" s="10">
         <v>16</v>
       </c>
-      <c r="AS15" s="10">
-        <v>1</v>
-      </c>
       <c r="AT15" s="10">
         <v>1</v>
       </c>
       <c r="AU15" s="10">
-        <v>0</v>
-      </c>
-      <c r="AV15" s="14">
+        <v>1</v>
+      </c>
+      <c r="AV15" s="10">
+        <v>0</v>
+      </c>
+      <c r="AW15" s="14">
         <v>60</v>
       </c>
-      <c r="AW15" s="15" t="s">
+      <c r="AX15" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="AX15" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY15" s="14">
+      <c r="AY15" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ15" s="14">
         <v>50</v>
       </c>
-      <c r="AZ15" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD15" s="4" t="s">
+      <c r="BA15" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE15" s="4" t="s">
         <v>385</v>
       </c>
-      <c r="BE15" s="5" t="s">
+      <c r="BF15" s="5" t="s">
         <v>386</v>
       </c>
-      <c r="BF15" s="4" t="s">
+      <c r="BG15" s="4" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="16" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:60" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
         <v>304</v>
       </c>
@@ -8714,25 +8763,25 @@
         <v>0</v>
       </c>
       <c r="AA16" s="13">
+        <v>1</v>
+      </c>
+      <c r="AB16" s="13">
         <v>1150</v>
       </c>
-      <c r="AB16" s="13">
+      <c r="AC16" s="13">
         <v>85</v>
       </c>
-      <c r="AC16" s="13">
-        <v>0</v>
-      </c>
       <c r="AD16" s="13">
         <v>0</v>
       </c>
       <c r="AE16" s="13">
         <v>0</v>
       </c>
-      <c r="AF16" s="11">
-        <v>1</v>
+      <c r="AF16" s="13">
+        <v>0</v>
       </c>
       <c r="AG16" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH16" s="11">
         <v>0</v>
@@ -8755,47 +8804,50 @@
       <c r="AN16" s="11">
         <v>0</v>
       </c>
-      <c r="AQ16" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR16" s="10">
+      <c r="AO16" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR16" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS16" s="10">
         <v>21</v>
       </c>
-      <c r="AS16" s="10">
-        <v>1</v>
-      </c>
       <c r="AT16" s="10">
         <v>1</v>
       </c>
       <c r="AU16" s="10">
         <v>1</v>
       </c>
-      <c r="AV16" s="14">
+      <c r="AV16" s="10">
+        <v>1</v>
+      </c>
+      <c r="AW16" s="14">
         <v>60</v>
       </c>
-      <c r="AW16" s="15" t="s">
+      <c r="AX16" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="AX16" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY16" s="14">
+      <c r="AY16" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ16" s="14">
         <v>50</v>
       </c>
-      <c r="AZ16" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD16" s="4" t="s">
+      <c r="BA16" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE16" s="4" t="s">
         <v>388</v>
       </c>
-      <c r="BE16" s="5" t="s">
+      <c r="BF16" s="5" t="s">
         <v>389</v>
       </c>
-      <c r="BF16" s="4" t="s">
+      <c r="BG16" s="4" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="17" spans="1:58" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
         <v>304</v>
       </c>
@@ -8860,25 +8912,25 @@
         <v>0</v>
       </c>
       <c r="AA17" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB17" s="13">
         <v>1226</v>
       </c>
-      <c r="AB17" s="13">
+      <c r="AC17" s="13">
         <v>279</v>
       </c>
-      <c r="AC17" s="13">
-        <v>0</v>
-      </c>
       <c r="AD17" s="13">
         <v>0</v>
       </c>
       <c r="AE17" s="13">
         <v>0</v>
       </c>
-      <c r="AF17" s="11">
-        <v>1</v>
+      <c r="AF17" s="13">
+        <v>0</v>
       </c>
       <c r="AG17" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH17" s="11">
         <v>0</v>
@@ -8901,47 +8953,50 @@
       <c r="AN17" s="11">
         <v>0</v>
       </c>
-      <c r="AQ17" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR17" s="10">
+      <c r="AO17" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR17" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS17" s="10">
         <v>8</v>
       </c>
-      <c r="AS17" s="10">
-        <v>1</v>
-      </c>
       <c r="AT17" s="10">
         <v>1</v>
       </c>
       <c r="AU17" s="10">
-        <v>0</v>
-      </c>
-      <c r="AV17" s="14">
+        <v>1</v>
+      </c>
+      <c r="AV17" s="10">
+        <v>0</v>
+      </c>
+      <c r="AW17" s="14">
         <v>60</v>
       </c>
-      <c r="AW17" s="15" t="s">
+      <c r="AX17" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="AX17" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY17" s="14">
+      <c r="AY17" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ17" s="14">
         <v>50</v>
       </c>
-      <c r="AZ17" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD17" s="4" t="s">
+      <c r="BA17" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE17" s="4" t="s">
         <v>391</v>
       </c>
-      <c r="BE17" s="5" t="s">
+      <c r="BF17" s="5" t="s">
         <v>392</v>
       </c>
-      <c r="BF17" s="4" t="s">
+      <c r="BG17" s="4" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="18" spans="1:58" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
         <v>304</v>
       </c>
@@ -9006,26 +9061,26 @@
         <v>0</v>
       </c>
       <c r="AA18" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB18" s="13">
         <v>1325</v>
       </c>
-      <c r="AB18" s="13">
+      <c r="AC18" s="13">
         <v>330</v>
       </c>
-      <c r="AC18" s="13">
-        <v>0</v>
-      </c>
       <c r="AD18" s="13">
         <v>0</v>
       </c>
       <c r="AE18" s="13">
         <v>0</v>
       </c>
-      <c r="AF18" s="11">
+      <c r="AF18" s="13">
+        <v>0</v>
+      </c>
+      <c r="AG18" s="11">
         <v>2</v>
       </c>
-      <c r="AG18" s="11">
-        <v>0</v>
-      </c>
       <c r="AH18" s="11">
         <v>0</v>
       </c>
@@ -9047,47 +9102,50 @@
       <c r="AN18" s="11">
         <v>0</v>
       </c>
-      <c r="AQ18" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR18" s="10">
+      <c r="AO18" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR18" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS18" s="10">
         <v>9</v>
       </c>
-      <c r="AS18" s="10">
-        <v>1</v>
-      </c>
       <c r="AT18" s="10">
         <v>1</v>
       </c>
       <c r="AU18" s="10">
-        <v>0</v>
-      </c>
-      <c r="AV18" s="14">
+        <v>1</v>
+      </c>
+      <c r="AV18" s="10">
+        <v>0</v>
+      </c>
+      <c r="AW18" s="14">
         <v>60</v>
       </c>
-      <c r="AW18" s="15" t="s">
+      <c r="AX18" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="AX18" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY18" s="14">
+      <c r="AY18" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ18" s="14">
         <v>50</v>
       </c>
-      <c r="AZ18" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD18" s="4" t="s">
+      <c r="BA18" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE18" s="4" t="s">
         <v>394</v>
       </c>
-      <c r="BE18" s="5" t="s">
+      <c r="BF18" s="5" t="s">
         <v>395</v>
       </c>
-      <c r="BF18" s="4" t="s">
+      <c r="BG18" s="4" t="s">
         <v>396</v>
       </c>
     </row>
-    <row r="19" spans="1:58" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
         <v>304</v>
       </c>
@@ -9152,25 +9210,25 @@
         <v>0</v>
       </c>
       <c r="AA19" s="13">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AB19" s="13">
         <v>1141</v>
       </c>
-      <c r="AB19" s="13">
+      <c r="AC19" s="13">
         <v>95</v>
       </c>
-      <c r="AC19" s="13">
+      <c r="AD19" s="13">
         <v>15</v>
       </c>
-      <c r="AD19" s="13">
-        <v>0</v>
-      </c>
       <c r="AE19" s="13">
         <v>0</v>
       </c>
-      <c r="AF19" s="11">
-        <v>1</v>
+      <c r="AF19" s="13">
+        <v>0</v>
       </c>
       <c r="AG19" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH19" s="11">
         <v>0</v>
@@ -9193,47 +9251,50 @@
       <c r="AN19" s="11">
         <v>0</v>
       </c>
-      <c r="AQ19" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR19" s="10">
+      <c r="AO19" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR19" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS19" s="10">
         <v>28</v>
       </c>
-      <c r="AS19" s="10">
-        <v>1</v>
-      </c>
       <c r="AT19" s="10">
         <v>1</v>
       </c>
       <c r="AU19" s="10">
         <v>1</v>
       </c>
-      <c r="AV19" s="14">
+      <c r="AV19" s="10">
+        <v>1</v>
+      </c>
+      <c r="AW19" s="14">
         <v>66</v>
       </c>
-      <c r="AW19" s="15" t="s">
+      <c r="AX19" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="AX19" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY19" s="14">
+      <c r="AY19" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ19" s="14">
         <v>50</v>
       </c>
-      <c r="AZ19" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD19" s="4" t="s">
+      <c r="BA19" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE19" s="4" t="s">
         <v>397</v>
       </c>
-      <c r="BE19" s="5" t="s">
+      <c r="BF19" s="5" t="s">
         <v>398</v>
       </c>
-      <c r="BF19" s="4" t="s">
+      <c r="BG19" s="4" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="20" spans="1:58" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="s">
         <v>304</v>
       </c>
@@ -9298,26 +9359,26 @@
         <v>0</v>
       </c>
       <c r="AA20" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB20" s="13">
         <v>1653</v>
       </c>
-      <c r="AB20" s="13">
+      <c r="AC20" s="13">
         <v>282</v>
       </c>
-      <c r="AC20" s="13">
+      <c r="AD20" s="13">
         <v>10</v>
       </c>
-      <c r="AD20" s="13">
-        <v>0</v>
-      </c>
       <c r="AE20" s="13">
         <v>0</v>
       </c>
-      <c r="AF20" s="11">
+      <c r="AF20" s="13">
+        <v>0</v>
+      </c>
+      <c r="AG20" s="11">
         <v>2</v>
       </c>
-      <c r="AG20" s="11">
-        <v>0</v>
-      </c>
       <c r="AH20" s="11">
         <v>0</v>
       </c>
@@ -9339,47 +9400,50 @@
       <c r="AN20" s="11">
         <v>0</v>
       </c>
-      <c r="AQ20" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR20" s="10">
+      <c r="AO20" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR20" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS20" s="10">
         <v>14</v>
       </c>
-      <c r="AS20" s="10">
-        <v>1</v>
-      </c>
       <c r="AT20" s="10">
         <v>1</v>
       </c>
       <c r="AU20" s="10">
-        <v>0</v>
-      </c>
-      <c r="AV20" s="14">
+        <v>1</v>
+      </c>
+      <c r="AV20" s="10">
+        <v>0</v>
+      </c>
+      <c r="AW20" s="14">
         <v>66</v>
       </c>
-      <c r="AW20" s="15" t="s">
+      <c r="AX20" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="AX20" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY20" s="14">
+      <c r="AY20" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ20" s="14">
         <v>50</v>
       </c>
-      <c r="AZ20" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD20" s="4" t="s">
+      <c r="BA20" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE20" s="4" t="s">
         <v>400</v>
       </c>
-      <c r="BE20" s="5" t="s">
+      <c r="BF20" s="5" t="s">
         <v>401</v>
       </c>
-      <c r="BF20" s="4" t="s">
+      <c r="BG20" s="4" t="s">
         <v>402</v>
       </c>
     </row>
-    <row r="21" spans="1:58" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
         <v>304</v>
       </c>
@@ -9444,25 +9508,25 @@
         <v>0</v>
       </c>
       <c r="AA21" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB21" s="13">
         <v>935</v>
       </c>
-      <c r="AB21" s="13">
+      <c r="AC21" s="13">
         <v>83</v>
       </c>
-      <c r="AC21" s="13">
+      <c r="AD21" s="13">
         <v>15</v>
       </c>
-      <c r="AD21" s="13">
-        <v>0</v>
-      </c>
       <c r="AE21" s="13">
         <v>0</v>
       </c>
-      <c r="AF21" s="11">
-        <v>1</v>
+      <c r="AF21" s="13">
+        <v>0</v>
       </c>
       <c r="AG21" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH21" s="11">
         <v>0</v>
@@ -9485,47 +9549,50 @@
       <c r="AN21" s="11">
         <v>0</v>
       </c>
-      <c r="AQ21" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR21" s="10">
+      <c r="AO21" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR21" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS21" s="10">
         <v>10</v>
       </c>
-      <c r="AS21" s="10">
-        <v>1</v>
-      </c>
       <c r="AT21" s="10">
         <v>1</v>
       </c>
       <c r="AU21" s="10">
         <v>1</v>
       </c>
-      <c r="AV21" s="14">
+      <c r="AV21" s="10">
+        <v>1</v>
+      </c>
+      <c r="AW21" s="14">
         <v>60</v>
       </c>
-      <c r="AW21" s="15" t="s">
+      <c r="AX21" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="AX21" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY21" s="14">
+      <c r="AY21" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ21" s="14">
         <v>50</v>
       </c>
-      <c r="AZ21" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD21" s="4" t="s">
+      <c r="BA21" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE21" s="4" t="s">
         <v>403</v>
       </c>
-      <c r="BE21" s="5" t="s">
+      <c r="BF21" s="5" t="s">
         <v>404</v>
       </c>
-      <c r="BF21" s="4" t="s">
+      <c r="BG21" s="4" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="22" spans="1:58" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="s">
         <v>304</v>
       </c>
@@ -9590,26 +9657,26 @@
         <v>0</v>
       </c>
       <c r="AA22" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB22" s="13">
         <v>1858</v>
       </c>
-      <c r="AB22" s="13">
+      <c r="AC22" s="13">
         <v>245</v>
       </c>
-      <c r="AC22" s="13">
-        <v>0</v>
-      </c>
       <c r="AD22" s="13">
         <v>0</v>
       </c>
       <c r="AE22" s="13">
         <v>0</v>
       </c>
-      <c r="AF22" s="11">
+      <c r="AF22" s="13">
+        <v>0</v>
+      </c>
+      <c r="AG22" s="11">
         <v>2</v>
       </c>
-      <c r="AG22" s="11">
-        <v>0</v>
-      </c>
       <c r="AH22" s="11">
         <v>0</v>
       </c>
@@ -9631,47 +9698,50 @@
       <c r="AN22" s="11">
         <v>0</v>
       </c>
-      <c r="AQ22" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR22" s="10">
+      <c r="AO22" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR22" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS22" s="10">
         <v>17</v>
       </c>
-      <c r="AS22" s="10">
-        <v>1</v>
-      </c>
       <c r="AT22" s="10">
         <v>1</v>
       </c>
       <c r="AU22" s="10">
-        <v>0</v>
-      </c>
-      <c r="AV22" s="14">
+        <v>1</v>
+      </c>
+      <c r="AV22" s="10">
+        <v>0</v>
+      </c>
+      <c r="AW22" s="14">
         <v>66</v>
       </c>
-      <c r="AW22" s="15" t="s">
+      <c r="AX22" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="AX22" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY22" s="14">
+      <c r="AY22" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ22" s="14">
         <v>50</v>
       </c>
-      <c r="AZ22" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD22" s="4" t="s">
+      <c r="BA22" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE22" s="4" t="s">
         <v>406</v>
       </c>
-      <c r="BE22" s="5" t="s">
+      <c r="BF22" s="5" t="s">
         <v>407</v>
       </c>
-      <c r="BF22" s="4" t="s">
+      <c r="BG22" s="4" t="s">
         <v>408</v>
       </c>
     </row>
-    <row r="23" spans="1:58" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:59" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
         <v>304</v>
       </c>
@@ -9736,26 +9806,26 @@
         <v>0</v>
       </c>
       <c r="AA23" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB23" s="13">
         <v>1270</v>
       </c>
-      <c r="AB23" s="13">
+      <c r="AC23" s="13">
         <v>240</v>
       </c>
-      <c r="AC23" s="13">
-        <v>0</v>
-      </c>
       <c r="AD23" s="13">
         <v>0</v>
       </c>
       <c r="AE23" s="13">
         <v>0</v>
       </c>
-      <c r="AF23" s="11">
+      <c r="AF23" s="13">
+        <v>0</v>
+      </c>
+      <c r="AG23" s="11">
         <v>2</v>
       </c>
-      <c r="AG23" s="11">
-        <v>0</v>
-      </c>
       <c r="AH23" s="11">
         <v>0</v>
       </c>
@@ -9777,47 +9847,50 @@
       <c r="AN23" s="11">
         <v>0</v>
       </c>
-      <c r="AQ23" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR23" s="10">
+      <c r="AO23" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR23" s="11">
+        <v>1</v>
+      </c>
+      <c r="AS23" s="10">
         <v>9</v>
       </c>
-      <c r="AS23" s="10">
-        <v>1</v>
-      </c>
       <c r="AT23" s="10">
         <v>1</v>
       </c>
       <c r="AU23" s="10">
-        <v>0</v>
-      </c>
-      <c r="AV23" s="14">
+        <v>1</v>
+      </c>
+      <c r="AV23" s="10">
+        <v>0</v>
+      </c>
+      <c r="AW23" s="14">
         <v>60</v>
       </c>
-      <c r="AW23" s="15" t="s">
+      <c r="AX23" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="AX23" s="10">
-        <v>1</v>
-      </c>
-      <c r="AY23" s="14">
+      <c r="AY23" s="10">
+        <v>1</v>
+      </c>
+      <c r="AZ23" s="14">
         <v>50</v>
       </c>
-      <c r="AZ23" s="10">
-        <v>1</v>
-      </c>
-      <c r="BD23" s="4" t="s">
+      <c r="BA23" s="10">
+        <v>1</v>
+      </c>
+      <c r="BE23" s="4" t="s">
         <v>409</v>
       </c>
-      <c r="BE23" s="5" t="s">
+      <c r="BF23" s="5" t="s">
         <v>410</v>
       </c>
-      <c r="BF23" s="4" t="s">
+      <c r="BG23" s="4" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="24" spans="1:58" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A24" s="9" t="s">
         <v>61</v>
       </c>
@@ -9880,25 +9953,25 @@
         <v>0</v>
       </c>
       <c r="AA24" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB24" s="13">
         <v>5500</v>
       </c>
-      <c r="AB24" s="13">
+      <c r="AC24" s="13">
         <v>265</v>
       </c>
-      <c r="AC24" s="13">
-        <v>0</v>
-      </c>
       <c r="AD24" s="13">
         <v>0</v>
       </c>
       <c r="AE24" s="13">
         <v>0</v>
       </c>
-      <c r="AF24" s="11">
-        <v>1</v>
+      <c r="AF24" s="13">
+        <v>0</v>
       </c>
       <c r="AG24" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH24" s="11">
         <v>0</v>
@@ -9921,29 +9994,32 @@
       <c r="AN24" s="11">
         <v>0</v>
       </c>
-      <c r="AQ24" s="11">
-        <v>0</v>
-      </c>
-      <c r="BA24" s="13">
+      <c r="AO24" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR24" s="11">
+        <v>0</v>
+      </c>
+      <c r="BB24" s="13">
         <v>0.5</v>
       </c>
-      <c r="BB24" s="11">
-        <v>1</v>
-      </c>
       <c r="BC24" s="11">
-        <v>0</v>
-      </c>
-      <c r="BD24" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="BD24" s="11">
+        <v>0</v>
+      </c>
+      <c r="BE24" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="BE24" s="5" t="s">
+      <c r="BF24" s="5" t="s">
         <v>294</v>
       </c>
-      <c r="BF24" s="4" t="s">
+      <c r="BG24" s="4" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="25" spans="1:58" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
         <v>61</v>
       </c>
@@ -10006,25 +10082,25 @@
         <v>0</v>
       </c>
       <c r="AA25" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB25" s="13">
         <v>4590</v>
       </c>
-      <c r="AB25" s="13">
+      <c r="AC25" s="13">
         <v>185</v>
       </c>
-      <c r="AC25" s="13">
-        <v>0</v>
-      </c>
       <c r="AD25" s="13">
         <v>0</v>
       </c>
       <c r="AE25" s="13">
         <v>0</v>
       </c>
-      <c r="AF25" s="11">
-        <v>1</v>
+      <c r="AF25" s="13">
+        <v>0</v>
       </c>
       <c r="AG25" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH25" s="11">
         <v>0</v>
@@ -10047,29 +10123,32 @@
       <c r="AN25" s="11">
         <v>0</v>
       </c>
-      <c r="AQ25" s="11">
-        <v>0</v>
-      </c>
-      <c r="BA25" s="13">
+      <c r="AO25" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR25" s="11">
+        <v>0</v>
+      </c>
+      <c r="BB25" s="13">
         <v>0.45</v>
       </c>
-      <c r="BB25" s="11">
-        <v>1</v>
-      </c>
       <c r="BC25" s="11">
-        <v>0</v>
-      </c>
-      <c r="BD25" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="BD25" s="11">
+        <v>0</v>
+      </c>
+      <c r="BE25" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="BE25" s="5" t="s">
+      <c r="BF25" s="5" t="s">
         <v>295</v>
       </c>
-      <c r="BF25" s="4" t="s">
+      <c r="BG25" s="4" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="26" spans="1:58" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
         <v>61</v>
       </c>
@@ -10129,25 +10208,25 @@
         <v>0</v>
       </c>
       <c r="AA26" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB26" s="13">
         <v>12000</v>
       </c>
-      <c r="AB26" s="13">
+      <c r="AC26" s="13">
         <v>325</v>
       </c>
-      <c r="AC26" s="13">
+      <c r="AD26" s="13">
         <v>10</v>
       </c>
-      <c r="AD26" s="13">
-        <v>0</v>
-      </c>
       <c r="AE26" s="13">
         <v>0</v>
       </c>
-      <c r="AF26" s="11">
-        <v>1</v>
+      <c r="AF26" s="13">
+        <v>0</v>
       </c>
       <c r="AG26" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH26" s="11">
         <v>0</v>
@@ -10170,29 +10249,32 @@
       <c r="AN26" s="11">
         <v>0</v>
       </c>
-      <c r="AQ26" s="11">
-        <v>0</v>
-      </c>
-      <c r="BA26" s="13">
+      <c r="AO26" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR26" s="11">
+        <v>0</v>
+      </c>
+      <c r="BB26" s="13">
         <v>0.4</v>
       </c>
-      <c r="BB26" s="11">
-        <v>1</v>
-      </c>
       <c r="BC26" s="11">
-        <v>0</v>
-      </c>
-      <c r="BD26" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="BD26" s="11">
+        <v>0</v>
+      </c>
+      <c r="BE26" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="BE26" s="5" t="s">
+      <c r="BF26" s="5" t="s">
         <v>303</v>
       </c>
-      <c r="BF26" s="4" t="s">
+      <c r="BG26" s="4" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="27" spans="1:58" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
         <v>61</v>
       </c>
@@ -10255,25 +10337,25 @@
         <v>0</v>
       </c>
       <c r="AA27" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB27" s="13">
         <v>12500</v>
       </c>
-      <c r="AB27" s="13">
+      <c r="AC27" s="13">
         <v>375</v>
       </c>
-      <c r="AC27" s="13">
+      <c r="AD27" s="13">
         <v>50</v>
       </c>
-      <c r="AD27" s="13">
-        <v>0</v>
-      </c>
       <c r="AE27" s="13">
         <v>0</v>
       </c>
-      <c r="AF27" s="11">
-        <v>1</v>
+      <c r="AF27" s="13">
+        <v>0</v>
       </c>
       <c r="AG27" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH27" s="11">
         <v>0</v>
@@ -10296,26 +10378,29 @@
       <c r="AN27" s="11">
         <v>0</v>
       </c>
-      <c r="AQ27" s="11">
-        <v>0</v>
-      </c>
-      <c r="BA27" s="13">
+      <c r="AO27" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR27" s="11">
+        <v>0</v>
+      </c>
+      <c r="BB27" s="13">
         <v>0.25</v>
       </c>
-      <c r="BB27" s="11">
-        <v>1</v>
-      </c>
       <c r="BC27" s="11">
-        <v>0</v>
-      </c>
-      <c r="BD27" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="BD27" s="11">
+        <v>0</v>
+      </c>
+      <c r="BE27" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="BE27" s="5" t="s">
+      <c r="BF27" s="5" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="28" spans="1:58" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
         <v>61</v>
       </c>
@@ -10375,25 +10460,25 @@
         <v>0</v>
       </c>
       <c r="AA28" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB28" s="13">
         <v>1235</v>
       </c>
-      <c r="AB28" s="13">
+      <c r="AC28" s="13">
         <v>65</v>
       </c>
-      <c r="AC28" s="13">
+      <c r="AD28" s="13">
         <v>5</v>
       </c>
-      <c r="AD28" s="13">
-        <v>0</v>
-      </c>
       <c r="AE28" s="13">
         <v>0</v>
       </c>
-      <c r="AF28" s="11">
-        <v>1</v>
+      <c r="AF28" s="13">
+        <v>0</v>
       </c>
       <c r="AG28" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH28" s="11">
         <v>0</v>
@@ -10416,29 +10501,32 @@
       <c r="AN28" s="11">
         <v>0</v>
       </c>
-      <c r="AQ28" s="11">
-        <v>0</v>
-      </c>
-      <c r="BA28" s="13">
-        <v>0</v>
-      </c>
-      <c r="BB28" s="11">
-        <v>1</v>
+      <c r="AO28" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR28" s="11">
+        <v>0</v>
+      </c>
+      <c r="BB28" s="13">
+        <v>0</v>
       </c>
       <c r="BC28" s="11">
-        <v>0</v>
-      </c>
-      <c r="BD28" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="BD28" s="11">
+        <v>0</v>
+      </c>
+      <c r="BE28" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="BE28" s="5" t="s">
+      <c r="BF28" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="BF28" s="4" t="s">
+      <c r="BG28" s="4" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="29" spans="1:58" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
         <v>61</v>
       </c>
@@ -10498,25 +10586,25 @@
         <v>0</v>
       </c>
       <c r="AA29" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB29" s="13">
         <v>3600</v>
       </c>
-      <c r="AB29" s="13">
+      <c r="AC29" s="13">
         <v>150</v>
       </c>
-      <c r="AC29" s="13">
+      <c r="AD29" s="13">
         <v>5</v>
       </c>
-      <c r="AD29" s="13">
-        <v>0</v>
-      </c>
       <c r="AE29" s="13">
         <v>0</v>
       </c>
-      <c r="AF29" s="11">
-        <v>1</v>
+      <c r="AF29" s="13">
+        <v>0</v>
       </c>
       <c r="AG29" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH29" s="11">
         <v>0</v>
@@ -10539,35 +10627,38 @@
       <c r="AN29" s="11">
         <v>0</v>
       </c>
-      <c r="AO29" s="12" t="s">
+      <c r="AO29" s="11">
+        <v>0</v>
+      </c>
+      <c r="AP29" s="12" t="s">
         <v>191</v>
       </c>
-      <c r="AP29" s="11" t="s">
+      <c r="AQ29" s="11" t="s">
         <v>179</v>
       </c>
-      <c r="AQ29" s="11">
-        <v>0</v>
-      </c>
-      <c r="BA29" s="13">
-        <v>0</v>
-      </c>
-      <c r="BB29" s="11">
-        <v>1</v>
+      <c r="AR29" s="11">
+        <v>0</v>
+      </c>
+      <c r="BB29" s="13">
+        <v>0</v>
       </c>
       <c r="BC29" s="11">
-        <v>0</v>
-      </c>
-      <c r="BD29" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="BD29" s="11">
+        <v>0</v>
+      </c>
+      <c r="BE29" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="BE29" s="5" t="s">
+      <c r="BF29" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="BF29" s="4" t="s">
+      <c r="BG29" s="4" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="30" spans="1:58" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
         <v>61</v>
       </c>
@@ -10627,25 +10718,25 @@
         <v>0</v>
       </c>
       <c r="AA30" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB30" s="13">
         <v>6900</v>
       </c>
-      <c r="AB30" s="13">
+      <c r="AC30" s="13">
         <v>235</v>
       </c>
-      <c r="AC30" s="13">
+      <c r="AD30" s="13">
         <v>5</v>
       </c>
-      <c r="AD30" s="13">
-        <v>0</v>
-      </c>
       <c r="AE30" s="13">
         <v>0</v>
       </c>
-      <c r="AF30" s="11">
-        <v>1</v>
+      <c r="AF30" s="13">
+        <v>0</v>
       </c>
       <c r="AG30" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH30" s="11">
         <v>0</v>
@@ -10668,35 +10759,38 @@
       <c r="AN30" s="11">
         <v>0</v>
       </c>
-      <c r="AO30" s="12" t="s">
+      <c r="AO30" s="11">
+        <v>0</v>
+      </c>
+      <c r="AP30" s="12" t="s">
         <v>192</v>
       </c>
-      <c r="AP30" s="11" t="s">
+      <c r="AQ30" s="11" t="s">
         <v>179</v>
       </c>
-      <c r="AQ30" s="11">
-        <v>0</v>
-      </c>
-      <c r="BA30" s="13">
-        <v>0</v>
-      </c>
-      <c r="BB30" s="11">
-        <v>1</v>
+      <c r="AR30" s="11">
+        <v>0</v>
+      </c>
+      <c r="BB30" s="13">
+        <v>0</v>
       </c>
       <c r="BC30" s="11">
-        <v>0</v>
-      </c>
-      <c r="BD30" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="BD30" s="11">
+        <v>0</v>
+      </c>
+      <c r="BE30" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="BE30" s="5" t="s">
+      <c r="BF30" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="BF30" s="4" t="s">
+      <c r="BG30" s="4" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="31" spans="1:58" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A31" s="9" t="s">
         <v>61</v>
       </c>
@@ -10753,25 +10847,25 @@
         <v>0</v>
       </c>
       <c r="AA31" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB31" s="13">
         <v>5000</v>
       </c>
-      <c r="AB31" s="13">
+      <c r="AC31" s="13">
         <v>500</v>
       </c>
-      <c r="AC31" s="13">
+      <c r="AD31" s="13">
         <v>50</v>
       </c>
-      <c r="AD31" s="13">
-        <v>0</v>
-      </c>
       <c r="AE31" s="13">
         <v>0</v>
       </c>
-      <c r="AF31" s="11">
-        <v>1</v>
+      <c r="AF31" s="13">
+        <v>0</v>
       </c>
       <c r="AG31" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH31" s="11">
         <v>0</v>
@@ -10794,26 +10888,29 @@
       <c r="AN31" s="11">
         <v>0</v>
       </c>
-      <c r="AQ31" s="11">
-        <v>0</v>
-      </c>
-      <c r="BA31" s="13">
+      <c r="AO31" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR31" s="11">
+        <v>0</v>
+      </c>
+      <c r="BB31" s="13">
         <v>0.45</v>
       </c>
-      <c r="BB31" s="11">
+      <c r="BC31" s="11">
         <v>2</v>
       </c>
-      <c r="BC31" s="11">
-        <v>0</v>
-      </c>
-      <c r="BD31" s="4" t="s">
+      <c r="BD31" s="11">
+        <v>0</v>
+      </c>
+      <c r="BE31" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="BE31" s="5" t="s">
+      <c r="BF31" s="5" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="32" spans="1:58" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A32" s="9" t="s">
         <v>61</v>
       </c>
@@ -10873,11 +10970,11 @@
         <v>0</v>
       </c>
       <c r="AA32" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB32" s="13">
         <v>100</v>
       </c>
-      <c r="AB32" s="13">
-        <v>0</v>
-      </c>
       <c r="AC32" s="13">
         <v>0</v>
       </c>
@@ -10887,7 +10984,7 @@
       <c r="AE32" s="13">
         <v>0</v>
       </c>
-      <c r="AF32" s="11">
+      <c r="AF32" s="13">
         <v>0</v>
       </c>
       <c r="AG32" s="11">
@@ -10914,17 +11011,17 @@
       <c r="AN32" s="11">
         <v>0</v>
       </c>
-      <c r="AO32" s="12" t="s">
+      <c r="AO32" s="11">
+        <v>0</v>
+      </c>
+      <c r="AP32" s="12" t="s">
         <v>193</v>
       </c>
-      <c r="AP32" s="11" t="s">
+      <c r="AQ32" s="11" t="s">
         <v>178</v>
       </c>
-      <c r="AQ32" s="11">
-        <v>1</v>
-      </c>
-      <c r="AR32" s="10">
-        <v>0</v>
+      <c r="AR32" s="11">
+        <v>1</v>
       </c>
       <c r="AS32" s="10">
         <v>0</v>
@@ -10935,29 +11032,32 @@
       <c r="AU32" s="10">
         <v>0</v>
       </c>
-      <c r="AV32" s="14">
-        <v>0</v>
-      </c>
-      <c r="AW32" s="15" t="s">
+      <c r="AV32" s="10">
+        <v>0</v>
+      </c>
+      <c r="AW32" s="14">
+        <v>0</v>
+      </c>
+      <c r="AX32" s="15" t="s">
         <v>195</v>
       </c>
-      <c r="AX32" s="10">
-        <v>0</v>
-      </c>
-      <c r="AY32" s="14">
-        <v>0</v>
-      </c>
-      <c r="AZ32" s="10">
-        <v>0</v>
-      </c>
-      <c r="BD32" s="4" t="s">
+      <c r="AY32" s="10">
+        <v>0</v>
+      </c>
+      <c r="AZ32" s="14">
+        <v>0</v>
+      </c>
+      <c r="BA32" s="10">
+        <v>0</v>
+      </c>
+      <c r="BE32" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="BE32" s="5" t="s">
+      <c r="BF32" s="5" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="33" spans="1:58" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A33" s="9" t="s">
         <v>61</v>
       </c>
@@ -11020,28 +11120,28 @@
         <v>0</v>
       </c>
       <c r="AA33" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB33" s="13">
         <v>32500</v>
       </c>
-      <c r="AB33" s="13">
+      <c r="AC33" s="13">
         <v>700</v>
       </c>
-      <c r="AC33" s="13">
+      <c r="AD33" s="13">
         <v>50</v>
       </c>
-      <c r="AD33" s="13">
-        <v>0</v>
-      </c>
       <c r="AE33" s="13">
         <v>0</v>
       </c>
-      <c r="AF33" s="11">
-        <v>1</v>
+      <c r="AF33" s="13">
+        <v>0</v>
       </c>
       <c r="AG33" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH33" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI33" s="11">
         <v>1</v>
@@ -11061,26 +11161,29 @@
       <c r="AN33" s="11">
         <v>1</v>
       </c>
-      <c r="AQ33" s="11">
-        <v>0</v>
-      </c>
-      <c r="BA33" s="13">
+      <c r="AO33" s="11">
+        <v>1</v>
+      </c>
+      <c r="AR33" s="11">
+        <v>0</v>
+      </c>
+      <c r="BB33" s="13">
         <v>0.3</v>
       </c>
-      <c r="BB33" s="11">
+      <c r="BC33" s="11">
         <v>7</v>
       </c>
-      <c r="BC33" s="11">
-        <v>0</v>
-      </c>
-      <c r="BD33" s="4" t="s">
+      <c r="BD33" s="11">
+        <v>0</v>
+      </c>
+      <c r="BE33" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="BE33" s="5" t="s">
+      <c r="BF33" s="5" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="34" spans="1:58" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
         <v>171</v>
       </c>
@@ -11125,11 +11228,11 @@
         <v>0</v>
       </c>
       <c r="AA34" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB34" s="13">
         <v>100</v>
       </c>
-      <c r="AB34" s="13">
-        <v>0</v>
-      </c>
       <c r="AC34" s="13">
         <v>0</v>
       </c>
@@ -11139,7 +11242,7 @@
       <c r="AE34" s="13">
         <v>0</v>
       </c>
-      <c r="AF34" s="11">
+      <c r="AF34" s="13">
         <v>0</v>
       </c>
       <c r="AG34" s="11">
@@ -11166,21 +11269,24 @@
       <c r="AN34" s="11">
         <v>0</v>
       </c>
-      <c r="AQ34" s="11">
-        <v>0</v>
-      </c>
-      <c r="BD34" s="4" t="s">
+      <c r="AO34" s="11">
+        <v>0</v>
+      </c>
+      <c r="AR34" s="11">
+        <v>0</v>
+      </c>
+      <c r="BE34" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="BE34" s="5" t="s">
+      <c r="BF34" s="5" t="s">
         <v>301</v>
       </c>
-      <c r="BF34" s="4" t="s">
+      <c r="BG34" s="4" t="s">
         <v>267</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:BC4" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A4:BD4" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
打包修复与退出确认：清理 Unity.Plastic/Codice/UnityEditorInternal 误 using 并统一标准 Newtonsoft.Json（XLSX2DataAsset、ComponentConfig 等6文件）；TerminalPanel 关卡列表改 Resources.LoadAll+按名排序，去除运行时 Assets/ 目录枚举；HomePanel 新增 CloseGame 按钮与 Esc 监听（面板栈顶期间），唤起确认弹窗后退出游戏；上调四类敌人 MaxHp 并微调 MC-4 creeper 波次间隔（1→1.2），同步 EntityAttributes.xlsx；LevelMessagePanel/CharacterSelectPanel 布局微调；MSYH/MSYHBD 字体图集扩充、LiberationSans Fallback 精简；BuildSettings 加入 SampleScene，UnityConnect 启用与 PlayerSettings 序列化刷新
</commit_message>
<xml_diff>
--- a/Assets/DataTools/EntityAttributes.xlsx
+++ b/Assets/DataTools/EntityAttributes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Unity\projects\TD\Assets\DataTools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D4F9535-0E9F-4D51-B86E-1179F629A337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B591D754-8391-4297-B9B2-9FA7CE2F8FFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3450" yWindow="340" windowWidth="19640" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9955,7 +9955,7 @@
         <v>0</v>
       </c>
       <c r="AB24" s="13">
-        <v>5500</v>
+        <v>5960</v>
       </c>
       <c r="AC24" s="13">
         <v>265</v>
@@ -10084,7 +10084,7 @@
         <v>0</v>
       </c>
       <c r="AB25" s="13">
-        <v>4590</v>
+        <v>5090</v>
       </c>
       <c r="AC25" s="13">
         <v>185</v>
@@ -10210,7 +10210,7 @@
         <v>0</v>
       </c>
       <c r="AB26" s="13">
-        <v>12000</v>
+        <v>12500</v>
       </c>
       <c r="AC26" s="13">
         <v>325</v>
@@ -10339,7 +10339,7 @@
         <v>0</v>
       </c>
       <c r="AB27" s="13">
-        <v>12500</v>
+        <v>13000</v>
       </c>
       <c r="AC27" s="13">
         <v>375</v>

</xml_diff>